<commit_message>
Backfill 00992A holdings 2026-05-28 to 2026-05-29
</commit_message>
<xml_diff>
--- a/data/raw/00992A_portfolio_20260529.xlsx
+++ b/data/raw/00992A_portfolio_20260529.xlsx
@@ -384,7 +384,7 @@
         <v>基金淨資產價值(元)</v>
       </c>
       <c r="B1" t="str">
-        <v>TWD 51,376,997,525</v>
+        <v>TWD 50,734,871,196</v>
       </c>
     </row>
     <row r="2">
@@ -392,7 +392,7 @@
         <v>每受益權單位淨資產價值(元)-台幣交易</v>
       </c>
       <c r="B2" t="str">
-        <v>TWD 18.42</v>
+        <v>TWD 18.07</v>
       </c>
     </row>
     <row r="3">
@@ -400,7 +400,7 @@
         <v>已發行受益權單位總數-台幣交易</v>
       </c>
       <c r="B3" t="str">
-        <v>2,788,455,000</v>
+        <v>2,807,455,000</v>
       </c>
     </row>
   </sheetData>
@@ -436,7 +436,7 @@
         <v>台積電</v>
       </c>
       <c r="C2" t="str">
-        <v>8.07%</v>
+        <v>7.97%</v>
       </c>
       <c r="D2" t="str">
         <v>1,761,000</v>
@@ -444,30 +444,30 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2383</v>
+        <v>3037</v>
       </c>
       <c r="B3" t="str">
-        <v>台光電</v>
+        <v>欣興</v>
       </c>
       <c r="C3" t="str">
-        <v>6.34%</v>
+        <v>5.86%</v>
       </c>
       <c r="D3" t="str">
-        <v>636,000</v>
+        <v>2,902,000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>3037</v>
+        <v>2383</v>
       </c>
       <c r="B4" t="str">
-        <v>欣興</v>
+        <v>台光電</v>
       </c>
       <c r="C4" t="str">
-        <v>5.96%</v>
+        <v>5.34%</v>
       </c>
       <c r="D4" t="str">
-        <v>2,902,000</v>
+        <v>536,000</v>
       </c>
     </row>
     <row r="5">
@@ -478,7 +478,7 @@
         <v>智邦</v>
       </c>
       <c r="C5" t="str">
-        <v>4.79%</v>
+        <v>4.86%</v>
       </c>
       <c r="D5" t="str">
         <v>1,012,000</v>
@@ -486,30 +486,30 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>6669</v>
+        <v>6223</v>
       </c>
       <c r="B6" t="str">
-        <v>緯穎</v>
+        <v>旺矽</v>
       </c>
       <c r="C6" t="str">
-        <v>4.24%</v>
+        <v>3.95%</v>
       </c>
       <c r="D6" t="str">
-        <v>400,000</v>
+        <v>339,000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>6223</v>
+        <v>6669</v>
       </c>
       <c r="B7" t="str">
-        <v>旺矽</v>
+        <v>緯穎</v>
       </c>
       <c r="C7" t="str">
-        <v>3.93%</v>
+        <v>3.9%</v>
       </c>
       <c r="D7" t="str">
-        <v>339,000</v>
+        <v>400,000</v>
       </c>
     </row>
     <row r="8">
@@ -520,7 +520,7 @@
         <v>高力</v>
       </c>
       <c r="C8" t="str">
-        <v>3.55%</v>
+        <v>3.61%</v>
       </c>
       <c r="D8" t="str">
         <v>1,674,000</v>
@@ -534,7 +534,7 @@
         <v>聯發科</v>
       </c>
       <c r="C9" t="str">
-        <v>3.46%</v>
+        <v>3.58%</v>
       </c>
       <c r="D9" t="str">
         <v>412,000</v>
@@ -542,30 +542,30 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>3017</v>
+        <v>3443</v>
       </c>
       <c r="B10" t="str">
-        <v>奇鋐</v>
+        <v>創意</v>
       </c>
       <c r="C10" t="str">
-        <v>3.38%</v>
+        <v>3.26%</v>
       </c>
       <c r="D10" t="str">
-        <v>651,000</v>
+        <v>360,000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>3443</v>
+        <v>3105</v>
       </c>
       <c r="B11" t="str">
-        <v>創意</v>
+        <v>穩懋</v>
       </c>
       <c r="C11" t="str">
-        <v>3.27%</v>
+        <v>3.16%</v>
       </c>
       <c r="D11" t="str">
-        <v>360,000</v>
+        <v>3,033,000</v>
       </c>
     </row>
     <row r="12">
@@ -576,7 +576,7 @@
         <v>川湖</v>
       </c>
       <c r="C12" t="str">
-        <v>3.18%</v>
+        <v>2.99%</v>
       </c>
       <c r="D12" t="str">
         <v>323,000</v>
@@ -590,7 +590,7 @@
         <v>貿聯-KY</v>
       </c>
       <c r="C13" t="str">
-        <v>2.71%</v>
+        <v>2.78%</v>
       </c>
       <c r="D13" t="str">
         <v>667,000</v>
@@ -604,7 +604,7 @@
         <v>穎崴</v>
       </c>
       <c r="C14" t="str">
-        <v>2.55%</v>
+        <v>2.71%</v>
       </c>
       <c r="D14" t="str">
         <v>151,000</v>
@@ -612,44 +612,44 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>3661</v>
+        <v>3017</v>
       </c>
       <c r="B15" t="str">
-        <v>世芯-KY</v>
+        <v>奇鋐</v>
       </c>
       <c r="C15" t="str">
-        <v>2.52%</v>
+        <v>2.55%</v>
       </c>
       <c r="D15" t="str">
-        <v>293,000</v>
+        <v>501,000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>8299</v>
+        <v>3661</v>
       </c>
       <c r="B16" t="str">
-        <v>群聯</v>
+        <v>世芯-KY</v>
       </c>
       <c r="C16" t="str">
-        <v>2.45%</v>
+        <v>2.48%</v>
       </c>
       <c r="D16" t="str">
-        <v>489,000</v>
+        <v>293,000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2455</v>
+        <v>8299</v>
       </c>
       <c r="B17" t="str">
-        <v>全新</v>
+        <v>群聯</v>
       </c>
       <c r="C17" t="str">
-        <v>2.32%</v>
+        <v>2.36%</v>
       </c>
       <c r="D17" t="str">
-        <v>2,827,000</v>
+        <v>489,000</v>
       </c>
     </row>
     <row r="18">
@@ -660,7 +660,7 @@
         <v>國巨*</v>
       </c>
       <c r="C18" t="str">
-        <v>2.3%</v>
+        <v>2.34%</v>
       </c>
       <c r="D18" t="str">
         <v>1,600,000</v>
@@ -668,72 +668,72 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>6584</v>
+        <v>2455</v>
       </c>
       <c r="B19" t="str">
-        <v>南俊國際</v>
+        <v>全新</v>
       </c>
       <c r="C19" t="str">
-        <v>2.15%</v>
+        <v>2.18%</v>
       </c>
       <c r="D19" t="str">
-        <v>1,485,000</v>
+        <v>2,827,000</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>6274</v>
+        <v>3711</v>
       </c>
       <c r="B20" t="str">
-        <v>台燿</v>
+        <v>日月光投控</v>
       </c>
       <c r="C20" t="str">
-        <v>2.09%</v>
+        <v>2.03%</v>
       </c>
       <c r="D20" t="str">
-        <v>636,000</v>
+        <v>1,640,000</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>3105</v>
+        <v>3081</v>
       </c>
       <c r="B21" t="str">
-        <v>穩懋</v>
+        <v>聯亞</v>
       </c>
       <c r="C21" t="str">
-        <v>2.09%</v>
+        <v>1.98%</v>
       </c>
       <c r="D21" t="str">
-        <v>2,033,000</v>
+        <v>380,000</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>3711</v>
+        <v>6584</v>
       </c>
       <c r="B22" t="str">
-        <v>日月光投控</v>
+        <v>南俊國際</v>
       </c>
       <c r="C22" t="str">
         <v>1.95%</v>
       </c>
       <c r="D22" t="str">
-        <v>1,640,000</v>
+        <v>1,437,000</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>3081</v>
+        <v>6274</v>
       </c>
       <c r="B23" t="str">
-        <v>聯亞</v>
+        <v>台燿</v>
       </c>
       <c r="C23" t="str">
         <v>1.93%</v>
       </c>
       <c r="D23" t="str">
-        <v>380,000</v>
+        <v>636,000</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         <v>南電</v>
       </c>
       <c r="C24" t="str">
-        <v>1.75%</v>
+        <v>1.77%</v>
       </c>
       <c r="D24" t="str">
         <v>1,058,000</v>
@@ -752,44 +752,44 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2368</v>
+        <v>6510</v>
       </c>
       <c r="B25" t="str">
-        <v>金像電</v>
+        <v>精測</v>
       </c>
       <c r="C25" t="str">
-        <v>1.72%</v>
+        <v>1.76%</v>
       </c>
       <c r="D25" t="str">
-        <v>669,000</v>
+        <v>272,000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2308</v>
+        <v>2368</v>
       </c>
       <c r="B26" t="str">
-        <v>台達電</v>
+        <v>金像電</v>
       </c>
       <c r="C26" t="str">
-        <v>1.7%</v>
+        <v>1.72%</v>
       </c>
       <c r="D26" t="str">
-        <v>357,000</v>
+        <v>669,000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>6510</v>
+        <v>2308</v>
       </c>
       <c r="B27" t="str">
-        <v>精測</v>
+        <v>台達電</v>
       </c>
       <c r="C27" t="str">
-        <v>1.66%</v>
+        <v>1.68%</v>
       </c>
       <c r="D27" t="str">
-        <v>272,000</v>
+        <v>357,000</v>
       </c>
     </row>
     <row r="28">
@@ -800,7 +800,7 @@
         <v>鴻勁</v>
       </c>
       <c r="C28" t="str">
-        <v>1.61%</v>
+        <v>1.52%</v>
       </c>
       <c r="D28" t="str">
         <v>100,000</v>
@@ -828,7 +828,7 @@
         <v>竑騰</v>
       </c>
       <c r="C30" t="str">
-        <v>1.32%</v>
+        <v>1.31%</v>
       </c>
       <c r="D30" t="str">
         <v>384,000</v>
@@ -842,7 +842,7 @@
         <v>信驊</v>
       </c>
       <c r="C31" t="str">
-        <v>1.11%</v>
+        <v>1.05%</v>
       </c>
       <c r="D31" t="str">
         <v>30,000</v>
@@ -856,7 +856,7 @@
         <v>致茂</v>
       </c>
       <c r="C32" t="str">
-        <v>1.02%</v>
+        <v>1.05%</v>
       </c>
       <c r="D32" t="str">
         <v>207,000</v>
@@ -864,114 +864,114 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>3583</v>
+        <v>4991</v>
       </c>
       <c r="B33" t="str">
-        <v>辛耘</v>
+        <v>環宇-KY</v>
       </c>
       <c r="C33" t="str">
-        <v>0.96%</v>
+        <v>0.8%</v>
       </c>
       <c r="D33" t="str">
-        <v>567,000</v>
+        <v>574,000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>4991</v>
+        <v>3189</v>
       </c>
       <c r="B34" t="str">
-        <v>環宇-KY</v>
+        <v>景碩</v>
       </c>
       <c r="C34" t="str">
-        <v>0.82%</v>
+        <v>0.65%</v>
       </c>
       <c r="D34" t="str">
-        <v>574,000</v>
+        <v>486,013</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>3189</v>
+        <v>6531</v>
       </c>
       <c r="B35" t="str">
-        <v>景碩</v>
+        <v>愛普*</v>
       </c>
       <c r="C35" t="str">
-        <v>0.69%</v>
+        <v>0.58%</v>
       </c>
       <c r="D35" t="str">
-        <v>486,013</v>
+        <v>271,000</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>6531</v>
+        <v>5289</v>
       </c>
       <c r="B36" t="str">
-        <v>愛普*</v>
+        <v>宜鼎</v>
       </c>
       <c r="C36" t="str">
-        <v>0.63%</v>
+        <v>0.53%</v>
       </c>
       <c r="D36" t="str">
-        <v>271,000</v>
+        <v>157,000</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>5289</v>
+        <v>2337</v>
       </c>
       <c r="B37" t="str">
-        <v>宜鼎</v>
+        <v>旺宏</v>
       </c>
       <c r="C37" t="str">
-        <v>0.55%</v>
+        <v>0.46%</v>
       </c>
       <c r="D37" t="str">
-        <v>157,000</v>
+        <v>1,465,000</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2337</v>
+        <v>8021</v>
       </c>
       <c r="B38" t="str">
-        <v>旺宏</v>
+        <v>尖點</v>
       </c>
       <c r="C38" t="str">
-        <v>0.47%</v>
+        <v>0.43%</v>
       </c>
       <c r="D38" t="str">
-        <v>1,465,000</v>
+        <v>518,000</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>8021</v>
+        <v>7734</v>
       </c>
       <c r="B39" t="str">
-        <v>尖點</v>
+        <v>印能科技</v>
       </c>
       <c r="C39" t="str">
-        <v>0.45%</v>
+        <v>0.43%</v>
       </c>
       <c r="D39" t="str">
-        <v>518,000</v>
+        <v>59,000</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>7734</v>
+        <v>6139</v>
       </c>
       <c r="B40" t="str">
-        <v>印能科技</v>
+        <v>亞翔</v>
       </c>
       <c r="C40" t="str">
-        <v>0.42%</v>
+        <v>0.39%</v>
       </c>
       <c r="D40" t="str">
-        <v>59,000</v>
+        <v>259,000</v>
       </c>
     </row>
     <row r="41">
@@ -982,7 +982,7 @@
         <v>富世達</v>
       </c>
       <c r="C41" t="str">
-        <v>0.42%</v>
+        <v>0.39%</v>
       </c>
       <c r="D41" t="str">
         <v>112,000</v>
@@ -990,72 +990,72 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>6139</v>
+        <v>3260</v>
       </c>
       <c r="B42" t="str">
-        <v>亞翔</v>
+        <v>威剛</v>
       </c>
       <c r="C42" t="str">
-        <v>0.4%</v>
+        <v>0.31%</v>
       </c>
       <c r="D42" t="str">
-        <v>259,000</v>
+        <v>393,000</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>3260</v>
+        <v>6442</v>
       </c>
       <c r="B43" t="str">
-        <v>威剛</v>
+        <v>光聖</v>
       </c>
       <c r="C43" t="str">
-        <v>0.32%</v>
+        <v>0.3%</v>
       </c>
       <c r="D43" t="str">
-        <v>393,000</v>
+        <v>80,000</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>6442</v>
+        <v>3533</v>
       </c>
       <c r="B44" t="str">
-        <v>光聖</v>
+        <v>嘉澤</v>
       </c>
       <c r="C44" t="str">
-        <v>0.29%</v>
+        <v>0.24%</v>
       </c>
       <c r="D44" t="str">
-        <v>80,000</v>
+        <v>48,000</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>3533</v>
+        <v>3491</v>
       </c>
       <c r="B45" t="str">
-        <v>嘉澤</v>
+        <v>昇達科</v>
       </c>
       <c r="C45" t="str">
-        <v>0.25%</v>
+        <v>0.19%</v>
       </c>
       <c r="D45" t="str">
-        <v>48,000</v>
+        <v>47,000</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>3491</v>
+        <v>3583</v>
       </c>
       <c r="B46" t="str">
-        <v>昇達科</v>
+        <v>辛耘</v>
       </c>
       <c r="C46" t="str">
-        <v>0.2%</v>
+        <v>0.06%</v>
       </c>
       <c r="D46" t="str">
-        <v>47,000</v>
+        <v>33,000</v>
       </c>
     </row>
   </sheetData>
@@ -1074,7 +1074,7 @@
         <v>應收付證券款</v>
       </c>
       <c r="B1" t="str">
-        <v>TWD 251,360,287.00</v>
+        <v>TWD 3,940,466,235.00</v>
       </c>
     </row>
     <row r="2">
@@ -1082,7 +1082,7 @@
         <v>應付贖回款</v>
       </c>
       <c r="B2" t="str">
-        <v>TWD -1,465,249,830.00</v>
+        <v>TWD -1,286,941,884.00</v>
       </c>
     </row>
     <row r="3">
@@ -1090,7 +1090,7 @@
         <v>現金</v>
       </c>
       <c r="B3" t="str">
-        <v>TWD 3,655,669,537.00</v>
+        <v>TWD 1,058,556,920.00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>